<commit_message>
Updated documentation after week 2 meeting
</commit_message>
<xml_diff>
--- a/Documentation/Week 2/Booked Hours/Booked_Hours_Christo.xlsx
+++ b/Documentation/Week 2/Booked Hours/Booked_Hours_Christo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uniwa-my.sharepoint.com/personal/24432207_student_uwa_edu_au/Documents/UWA - Student/2026_Sem2/CITS3200 - Professional Computing/Project/Repo/CITS3200_Project/Documentation/Week 2/Booked Hours/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="13_ncr:40009_{31A31D98-CA30-574B-8C94-F50C456CB544}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ADB0F1BA-E56C-47C4-A3CC-ED3B3B07D486}"/>
+  <xr:revisionPtr revIDLastSave="21" documentId="13_ncr:40009_{31A31D98-CA30-574B-8C94-F50C456CB544}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D145DF6E-0C46-46FA-9720-64135EF3C5A8}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="1920" yWindow="1920" windowWidth="17280" windowHeight="9960" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BookedHours" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="14">
   <si>
     <t>Wk</t>
   </si>
@@ -84,6 +84,12 @@
   </si>
   <si>
     <t>Researching group project requirements, getting familiar with project documentation, writing agenda</t>
+  </si>
+  <si>
+    <t>11:00AM</t>
+  </si>
+  <si>
+    <t>Team meeting</t>
   </si>
 </sst>
 </file>
@@ -303,6 +309,10 @@
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -313,6 +323,14 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -335,24 +353,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
   </cellXfs>
@@ -438,6 +444,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -770,7 +780,7 @@
     <col min="3" max="3" width="8.1796875" style="1" customWidth="1"/>
     <col min="4" max="4" width="10.26953125" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="8.81640625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="46.453125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="58.6328125" style="1" customWidth="1"/>
     <col min="7" max="7" width="9.36328125" style="1" customWidth="1"/>
     <col min="8" max="8" width="10.6328125" style="1"/>
     <col min="9" max="9" width="7.7265625" style="1" customWidth="1"/>
@@ -778,41 +788,41 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="70.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
-      <c r="H1" s="12"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="15"/>
     </row>
     <row r="2" spans="1:9" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="8" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="15" t="s">
+      <c r="A2" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="16"/>
-      <c r="D2" s="15" t="s">
+      <c r="C2" s="12"/>
+      <c r="D2" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="16"/>
-      <c r="F2" s="17" t="s">
+      <c r="E2" s="12"/>
+      <c r="F2" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="8" t="s">
+      <c r="G2" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="H2" s="13" t="s">
+      <c r="H2" s="16" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="13.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="9"/>
+      <c r="A3" s="10"/>
       <c r="B3" s="2" t="s">
         <v>2</v>
       </c>
@@ -825,9 +835,9 @@
       <c r="E3" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="18"/>
-      <c r="G3" s="9"/>
-      <c r="H3" s="14"/>
+      <c r="F3" s="19"/>
+      <c r="G3" s="10"/>
+      <c r="H3" s="17"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
@@ -836,7 +846,7 @@
       <c r="B4" s="4">
         <v>44770</v>
       </c>
-      <c r="C4" s="19" t="s">
+      <c r="C4" s="7" t="s">
         <v>9</v>
       </c>
       <c r="D4" s="4">
@@ -862,21 +872,33 @@
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="B5" s="4"/>
-      <c r="C5" s="5"/>
-      <c r="D5" s="4"/>
+      <c r="A5" s="1">
+        <v>2</v>
+      </c>
+      <c r="B5" s="4">
+        <v>44770</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" s="4">
+        <v>44770</v>
+      </c>
       <c r="E5" s="5"/>
-      <c r="G5" s="6" t="str">
+      <c r="F5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G5" s="6" t="e">
         <f t="shared" ref="G5:G30" si="0">IF(I5&gt;0,I5,IF(I5=0, " ", "ERROR"))</f>
-        <v xml:space="preserve"> </v>
+        <v>#VALUE!</v>
       </c>
       <c r="H5" s="1" t="e">
         <f>IF(AND(G5&lt;&gt;" ",G5&lt;&gt;"ERROR",H4&lt;&gt;" ", H4&lt;&gt;"ERROR"),G5+H4," ")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="I5" s="1">
+      <c r="I5" s="1" t="e">
         <f t="shared" ref="I5:I68" si="1">((D5+E5)-(B5+C5))*24</f>
-        <v>0</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
@@ -1330,24 +1352,24 @@
       </c>
     </row>
     <row r="31" spans="1:9" ht="15" x14ac:dyDescent="0.25">
-      <c r="A31" s="8" t="s">
-        <v>0</v>
-      </c>
-      <c r="B31" s="15" t="s">
+      <c r="A31" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="B31" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="C31" s="16"/>
-      <c r="D31" s="15" t="s">
+      <c r="C31" s="12"/>
+      <c r="D31" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="E31" s="16"/>
-      <c r="F31" s="7" t="s">
+      <c r="E31" s="12"/>
+      <c r="F31" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G31" s="7" t="s">
+      <c r="G31" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="H31" s="7" t="s">
+      <c r="H31" s="8" t="s">
         <v>6</v>
       </c>
       <c r="I31" s="1" t="e">
@@ -1356,7 +1378,7 @@
       </c>
     </row>
     <row r="32" spans="1:9" ht="15" x14ac:dyDescent="0.25">
-      <c r="A32" s="9"/>
+      <c r="A32" s="10"/>
       <c r="B32" s="2" t="s">
         <v>2</v>
       </c>
@@ -1369,9 +1391,9 @@
       <c r="E32" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="F32" s="7"/>
-      <c r="G32" s="7"/>
-      <c r="H32" s="7"/>
+      <c r="F32" s="8"/>
+      <c r="G32" s="8"/>
+      <c r="H32" s="8"/>
       <c r="I32" s="1" t="e">
         <f t="shared" si="1"/>
         <v>#VALUE!</v>
@@ -1939,24 +1961,24 @@
       </c>
     </row>
     <row r="65" spans="1:9" ht="15" x14ac:dyDescent="0.25">
-      <c r="A65" s="8" t="s">
-        <v>0</v>
-      </c>
-      <c r="B65" s="15" t="s">
+      <c r="A65" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="B65" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="C65" s="16"/>
-      <c r="D65" s="15" t="s">
+      <c r="C65" s="12"/>
+      <c r="D65" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="E65" s="16"/>
-      <c r="F65" s="7" t="s">
+      <c r="E65" s="12"/>
+      <c r="F65" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G65" s="7" t="s">
+      <c r="G65" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="H65" s="7" t="s">
+      <c r="H65" s="8" t="s">
         <v>6</v>
       </c>
       <c r="I65" s="1" t="e">
@@ -1965,7 +1987,7 @@
       </c>
     </row>
     <row r="66" spans="1:9" ht="15" x14ac:dyDescent="0.25">
-      <c r="A66" s="9"/>
+      <c r="A66" s="10"/>
       <c r="B66" s="2" t="s">
         <v>2</v>
       </c>
@@ -1978,9 +2000,9 @@
       <c r="E66" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="F66" s="7"/>
-      <c r="G66" s="7"/>
-      <c r="H66" s="7"/>
+      <c r="F66" s="8"/>
+      <c r="G66" s="8"/>
+      <c r="H66" s="8"/>
       <c r="I66" s="1" t="e">
         <f t="shared" si="1"/>
         <v>#VALUE!</v>
@@ -2435,24 +2457,24 @@
       </c>
     </row>
     <row r="99" spans="1:9" ht="15" x14ac:dyDescent="0.25">
-      <c r="A99" s="8" t="s">
-        <v>0</v>
-      </c>
-      <c r="B99" s="15" t="s">
+      <c r="A99" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="B99" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="C99" s="16"/>
-      <c r="D99" s="15" t="s">
+      <c r="C99" s="12"/>
+      <c r="D99" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="E99" s="16"/>
-      <c r="F99" s="7" t="s">
+      <c r="E99" s="12"/>
+      <c r="F99" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G99" s="7" t="s">
+      <c r="G99" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="H99" s="7" t="s">
+      <c r="H99" s="8" t="s">
         <v>6</v>
       </c>
       <c r="I99" s="1" t="e">
@@ -2461,7 +2483,7 @@
       </c>
     </row>
     <row r="100" spans="1:9" ht="15" x14ac:dyDescent="0.25">
-      <c r="A100" s="9"/>
+      <c r="A100" s="10"/>
       <c r="B100" s="2" t="s">
         <v>2</v>
       </c>
@@ -2474,9 +2496,9 @@
       <c r="E100" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="F100" s="7"/>
-      <c r="G100" s="7"/>
-      <c r="H100" s="7"/>
+      <c r="F100" s="8"/>
+      <c r="G100" s="8"/>
+      <c r="H100" s="8"/>
       <c r="I100" s="1" t="e">
         <f t="shared" si="7"/>
         <v>#VALUE!</v>
@@ -2932,18 +2954,6 @@
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="H99:H100"/>
-    <mergeCell ref="A99:A100"/>
-    <mergeCell ref="B99:C99"/>
-    <mergeCell ref="D99:E99"/>
-    <mergeCell ref="F99:F100"/>
-    <mergeCell ref="G99:G100"/>
-    <mergeCell ref="G65:G66"/>
-    <mergeCell ref="H65:H66"/>
-    <mergeCell ref="A65:A66"/>
-    <mergeCell ref="B65:C65"/>
-    <mergeCell ref="D65:E65"/>
-    <mergeCell ref="F65:F66"/>
     <mergeCell ref="H31:H32"/>
     <mergeCell ref="G2:G3"/>
     <mergeCell ref="A1:H1"/>
@@ -2957,6 +2967,18 @@
     <mergeCell ref="D31:E31"/>
     <mergeCell ref="F31:F32"/>
     <mergeCell ref="G31:G32"/>
+    <mergeCell ref="G65:G66"/>
+    <mergeCell ref="H65:H66"/>
+    <mergeCell ref="A65:A66"/>
+    <mergeCell ref="B65:C65"/>
+    <mergeCell ref="D65:E65"/>
+    <mergeCell ref="F65:F66"/>
+    <mergeCell ref="H99:H100"/>
+    <mergeCell ref="A99:A100"/>
+    <mergeCell ref="B99:C99"/>
+    <mergeCell ref="D99:E99"/>
+    <mergeCell ref="F99:F100"/>
+    <mergeCell ref="G99:G100"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.74803149606299213" right="0.74803149606299213" top="0.98425196850393704" bottom="0.98425196850393704" header="0.51181102362204722" footer="0.51181102362204722"/>

</xml_diff>

<commit_message>
Creation of Sprint 1 Deliverable Documents
</commit_message>
<xml_diff>
--- a/Documentation/Week 2/Booked Hours/Booked_Hours_Christo.xlsx
+++ b/Documentation/Week 2/Booked Hours/Booked_Hours_Christo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uniwa-my.sharepoint.com/personal/24432207_student_uwa_edu_au/Documents/UWA - Student/2026_Sem2/CITS3200 - Professional Computing/Project/Repo/CITS3200_Project/Documentation/Week 2/Booked Hours/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="25" documentId="13_ncr:40009_{31A31D98-CA30-574B-8C94-F50C456CB544}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5ED2E167-1226-49A0-BEE7-84D84FBB1580}"/>
+  <xr:revisionPtr revIDLastSave="32" documentId="13_ncr:40009_{31A31D98-CA30-574B-8C94-F50C456CB544}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2F95C330-0835-4D67-96EB-56517313C574}"/>
   <bookViews>
-    <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="20985" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3675" yWindow="3315" windowWidth="17280" windowHeight="9960" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BookedHours" sheetId="1" r:id="rId1"/>
@@ -312,6 +312,14 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" wrapText="1"/>
       <protection locked="0"/>
@@ -330,14 +338,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
@@ -431,6 +431,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -756,55 +760,55 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I132"/>
-  <sheetFormatPr defaultColWidth="10.6328125" defaultRowHeight="12.6" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="5.81640625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="10.36328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.6328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.36328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.6328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="46.453125" style="1" customWidth="1"/>
-    <col min="7" max="7" width="9.36328125" style="1" customWidth="1"/>
-    <col min="8" max="8" width="10.6328125" style="1"/>
-    <col min="9" max="9" width="10.6328125" style="1" hidden="1" customWidth="1"/>
-    <col min="10" max="16384" width="10.6328125" style="1"/>
+    <col min="1" max="1" width="5.875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="11.375" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.375" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="46.5" style="1" customWidth="1"/>
+    <col min="7" max="7" width="9.375" style="1" customWidth="1"/>
+    <col min="8" max="8" width="10.625" style="1"/>
+    <col min="9" max="9" width="10.625" style="1" hidden="1" customWidth="1"/>
+    <col min="10" max="16384" width="10.625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="70.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="10" t="s">
+    <row r="1" spans="1:9" ht="70.900000000000006" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
-      <c r="H1" s="12"/>
-    </row>
-    <row r="2" spans="1:9" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="14"/>
+    </row>
+    <row r="2" spans="1:9" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="16"/>
-      <c r="D2" s="15" t="s">
+      <c r="C2" s="11"/>
+      <c r="D2" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="16"/>
+      <c r="E2" s="11"/>
       <c r="F2" s="17" t="s">
         <v>5</v>
       </c>
       <c r="G2" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="H2" s="13" t="s">
+      <c r="H2" s="15" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="13.05" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" ht="13.15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="9"/>
       <c r="B3" s="2" t="s">
         <v>2</v>
@@ -820,7 +824,7 @@
       </c>
       <c r="F3" s="18"/>
       <c r="G3" s="9"/>
-      <c r="H3" s="14"/>
+      <c r="H3" s="16"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
@@ -887,21 +891,32 @@
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="B6" s="4"/>
-      <c r="C6" s="5"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="5"/>
-      <c r="G6" s="6" t="str">
+      <c r="A6" s="1">
+        <v>2</v>
+      </c>
+      <c r="B6" s="4">
+        <v>44770</v>
+      </c>
+      <c r="C6" s="5">
+        <v>0.64583333333333337</v>
+      </c>
+      <c r="D6" s="4">
+        <v>44770</v>
+      </c>
+      <c r="E6" s="5">
+        <v>0.67708333333333337</v>
+      </c>
+      <c r="G6" s="6">
         <f t="shared" si="0"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H6" s="1" t="str">
+        <v>0.75</v>
+      </c>
+      <c r="H6" s="1">
         <f t="shared" ref="H6:H30" si="2">IF(AND(G6&lt;&gt;" ",G6&lt;&gt;"ERROR",H5&lt;&gt;" ", H5&lt;&gt;"ERROR"),G6+H5," ")</f>
-        <v xml:space="preserve"> </v>
+        <v>3</v>
       </c>
       <c r="I6" s="1">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">
@@ -1336,18 +1351,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:9" ht="15" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:9" ht="15" x14ac:dyDescent="0.2">
       <c r="A31" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B31" s="15" t="s">
+      <c r="B31" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C31" s="16"/>
-      <c r="D31" s="15" t="s">
+      <c r="C31" s="11"/>
+      <c r="D31" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E31" s="16"/>
+      <c r="E31" s="11"/>
       <c r="F31" s="7" t="s">
         <v>5</v>
       </c>
@@ -1362,7 +1377,7 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="32" spans="1:9" ht="15" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:9" ht="15" x14ac:dyDescent="0.2">
       <c r="A32" s="9"/>
       <c r="B32" s="2" t="s">
         <v>2</v>
@@ -1945,18 +1960,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:9" ht="15" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:9" ht="15" x14ac:dyDescent="0.2">
       <c r="A65" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B65" s="15" t="s">
+      <c r="B65" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C65" s="16"/>
-      <c r="D65" s="15" t="s">
+      <c r="C65" s="11"/>
+      <c r="D65" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E65" s="16"/>
+      <c r="E65" s="11"/>
       <c r="F65" s="7" t="s">
         <v>5</v>
       </c>
@@ -1971,7 +1986,7 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="66" spans="1:9" ht="15" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:9" ht="15" x14ac:dyDescent="0.2">
       <c r="A66" s="9"/>
       <c r="B66" s="2" t="s">
         <v>2</v>
@@ -2441,18 +2456,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="1:9" ht="15" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:9" ht="15" x14ac:dyDescent="0.2">
       <c r="A99" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B99" s="15" t="s">
+      <c r="B99" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C99" s="16"/>
-      <c r="D99" s="15" t="s">
+      <c r="C99" s="11"/>
+      <c r="D99" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E99" s="16"/>
+      <c r="E99" s="11"/>
       <c r="F99" s="7" t="s">
         <v>5</v>
       </c>
@@ -2467,7 +2482,7 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="100" spans="1:9" ht="15" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:9" ht="15" x14ac:dyDescent="0.2">
       <c r="A100" s="9"/>
       <c r="B100" s="2" t="s">
         <v>2</v>
@@ -2939,18 +2954,6 @@
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="H99:H100"/>
-    <mergeCell ref="A99:A100"/>
-    <mergeCell ref="B99:C99"/>
-    <mergeCell ref="D99:E99"/>
-    <mergeCell ref="F99:F100"/>
-    <mergeCell ref="G99:G100"/>
-    <mergeCell ref="G65:G66"/>
-    <mergeCell ref="H65:H66"/>
-    <mergeCell ref="A65:A66"/>
-    <mergeCell ref="B65:C65"/>
-    <mergeCell ref="D65:E65"/>
-    <mergeCell ref="F65:F66"/>
     <mergeCell ref="H31:H32"/>
     <mergeCell ref="G2:G3"/>
     <mergeCell ref="A1:H1"/>
@@ -2964,6 +2967,18 @@
     <mergeCell ref="D31:E31"/>
     <mergeCell ref="F31:F32"/>
     <mergeCell ref="G31:G32"/>
+    <mergeCell ref="G65:G66"/>
+    <mergeCell ref="H65:H66"/>
+    <mergeCell ref="A65:A66"/>
+    <mergeCell ref="B65:C65"/>
+    <mergeCell ref="D65:E65"/>
+    <mergeCell ref="F65:F66"/>
+    <mergeCell ref="H99:H100"/>
+    <mergeCell ref="A99:A100"/>
+    <mergeCell ref="B99:C99"/>
+    <mergeCell ref="D99:E99"/>
+    <mergeCell ref="F99:F100"/>
+    <mergeCell ref="G99:G100"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.74803149606299213" right="0.74803149606299213" top="0.98425196850393704" bottom="0.98425196850393704" header="0.51181102362204722" footer="0.51181102362204722"/>
@@ -2975,7 +2990,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="12.6" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2987,7 +3002,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="12.6" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Timesheet and Booked Hours
- Corrected Booked Hours addition mistakes regarding time addition and added names at top of sheets
- Filled in Timesheet for this week
</commit_message>
<xml_diff>
--- a/Documentation/Week 2/Booked Hours/Booked_Hours_Christo.xlsx
+++ b/Documentation/Week 2/Booked Hours/Booked_Hours_Christo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uniwa-my.sharepoint.com/personal/24432207_student_uwa_edu_au/Documents/UWA - Student/2026_Sem2/CITS3200 - Professional Computing/Project/Repo/CITS3200_Project/Documentation/Week 2/Booked Hours/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="47" documentId="13_ncr:40009_{31A31D98-CA30-574B-8C94-F50C456CB544}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F1A04513-E903-4F09-AA11-A6EC5359DF83}"/>
+  <xr:revisionPtr revIDLastSave="53" documentId="13_ncr:40009_{31A31D98-CA30-574B-8C94-F50C456CB544}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0578D03B-2083-46EF-87C1-E8BDE6E000C8}"/>
   <bookViews>
-    <workbookView xWindow="624" yWindow="696" windowWidth="21600" windowHeight="11232" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BookedHours" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="15">
   <si>
     <t>Wk</t>
   </si>
@@ -90,6 +90,9 @@
   </si>
   <si>
     <t>Finishing meeting minutes</t>
+  </si>
+  <si>
+    <t>Filling in Team Timesheet</t>
   </si>
 </sst>
 </file>
@@ -442,6 +445,10 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -765,21 +772,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I132"/>
-  <sheetFormatPr defaultColWidth="10.625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.6328125" defaultRowHeight="12.6" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="5.875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="11.375" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.375" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.625" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="46.5" style="1" customWidth="1"/>
-    <col min="7" max="7" width="9.375" style="1" customWidth="1"/>
-    <col min="8" max="8" width="10.625" style="1"/>
-    <col min="9" max="9" width="10.625" style="1" hidden="1" customWidth="1"/>
-    <col min="10" max="16384" width="10.625" style="1"/>
+    <col min="1" max="1" width="5.90625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="11.36328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.6328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.36328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.6328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="46.453125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="9.36328125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="10.6328125" style="1"/>
+    <col min="9" max="9" width="10.6328125" style="1" hidden="1" customWidth="1"/>
+    <col min="10" max="16384" width="10.6328125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="70.900000000000006" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" ht="70.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>10</v>
       </c>
@@ -791,7 +798,7 @@
       <c r="G1" s="11"/>
       <c r="H1" s="12"/>
     </row>
-    <row r="2" spans="1:9" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:9" ht="16.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
         <v>0</v>
       </c>
@@ -813,7 +820,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="13.15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:9" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="9"/>
       <c r="B3" s="2" t="s">
         <v>2</v>
@@ -992,21 +999,35 @@
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="B9" s="4"/>
-      <c r="C9" s="5"/>
-      <c r="D9" s="4"/>
-      <c r="E9" s="5"/>
-      <c r="G9" s="6" t="str">
+      <c r="A9" s="1">
+        <v>2</v>
+      </c>
+      <c r="B9" s="4">
+        <v>44772</v>
+      </c>
+      <c r="C9" s="5">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="D9" s="4">
+        <v>44772</v>
+      </c>
+      <c r="E9" s="5">
+        <v>0.8125</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G9" s="6">
         <f t="shared" si="0"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H9" s="1" t="str">
+        <v>0.50000000005820766</v>
+      </c>
+      <c r="H9" s="1">
         <f t="shared" si="2"/>
-        <v xml:space="preserve"> </v>
+        <v>5.0000000000582077</v>
       </c>
       <c r="I9" s="1">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.50000000005820766</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.2">
@@ -1387,7 +1408,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:9" ht="15" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="A31" s="8" t="s">
         <v>0</v>
       </c>
@@ -1413,7 +1434,7 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="32" spans="1:9" ht="15" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="A32" s="9"/>
       <c r="B32" s="2" t="s">
         <v>2</v>
@@ -1996,7 +2017,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:9" ht="15" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="A65" s="8" t="s">
         <v>0</v>
       </c>
@@ -2022,7 +2043,7 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="66" spans="1:9" ht="15" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="A66" s="9"/>
       <c r="B66" s="2" t="s">
         <v>2</v>
@@ -2492,7 +2513,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="1:9" ht="15" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="A99" s="8" t="s">
         <v>0</v>
       </c>
@@ -2518,7 +2539,7 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="100" spans="1:9" ht="15" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="A100" s="9"/>
       <c r="B100" s="2" t="s">
         <v>2</v>
@@ -3026,7 +3047,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="12.6" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3038,7 +3059,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="12.6" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Sync documentation with main
</commit_message>
<xml_diff>
--- a/Documentation/Week 2/Booked Hours/Booked_Hours_Christo.xlsx
+++ b/Documentation/Week 2/Booked Hours/Booked_Hours_Christo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uniwa-my.sharepoint.com/personal/24432207_student_uwa_edu_au/Documents/UWA - Student/2026_Sem2/CITS3200 - Professional Computing/Project/Repo/CITS3200_Project/Documentation/Week 2/Booked Hours/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="53" documentId="13_ncr:40009_{31A31D98-CA30-574B-8C94-F50C456CB544}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0578D03B-2083-46EF-87C1-E8BDE6E000C8}"/>
+  <xr:revisionPtr revIDLastSave="25" documentId="13_ncr:40009_{31A31D98-CA30-574B-8C94-F50C456CB544}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5ED2E167-1226-49A0-BEE7-84D84FBB1580}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="20985" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BookedHours" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="11">
   <si>
     <t>Wk</t>
   </si>
@@ -81,18 +81,6 @@
       <t xml:space="preserve">
 Each time you do some work on the project, note the week number, start and end date and hour, plus a brief description of the activity. At the end of each week send a copy of the sheet as it currently stands to your group's manager for recording on the group TimeSheet. Date in the form DD/MM/YY and time as XX:YY (24hr clock)</t>
     </r>
-  </si>
-  <si>
-    <t>Writing up team documentation as well as researching project information</t>
-  </si>
-  <si>
-    <t>Client meeting</t>
-  </si>
-  <si>
-    <t>Finishing meeting minutes</t>
-  </si>
-  <si>
-    <t>Filling in Team Timesheet</t>
   </si>
 </sst>
 </file>
@@ -445,10 +433,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -774,10 +758,10 @@
   <dimension ref="A1:I132"/>
   <sheetFormatPr defaultColWidth="10.6328125" defaultRowHeight="12.6" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="5.90625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="11.36328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="5.81640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="10.36328125" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15.6328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.36328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.36328125" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="15.6328125" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="46.453125" style="1" customWidth="1"/>
     <col min="7" max="7" width="9.36328125" style="1" customWidth="1"/>
@@ -798,7 +782,7 @@
       <c r="G1" s="11"/>
       <c r="H1" s="12"/>
     </row>
-    <row r="2" spans="1:9" ht="16.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
         <v>0</v>
       </c>
@@ -820,7 +804,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" ht="13.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="9"/>
       <c r="B3" s="2" t="s">
         <v>2</v>
@@ -903,131 +887,75 @@
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A6" s="1">
-        <v>2</v>
-      </c>
-      <c r="B6" s="4">
-        <v>44770</v>
-      </c>
-      <c r="C6" s="5">
-        <v>0.64583333333333337</v>
-      </c>
-      <c r="D6" s="4">
-        <v>44770</v>
-      </c>
-      <c r="E6" s="5">
-        <v>0.67708333333333337</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="G6" s="6">
+      <c r="B6" s="4"/>
+      <c r="C6" s="5"/>
+      <c r="D6" s="4"/>
+      <c r="E6" s="5"/>
+      <c r="G6" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>0.75</v>
-      </c>
-      <c r="H6" s="1">
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H6" s="1" t="str">
         <f t="shared" ref="H6:H30" si="2">IF(AND(G6&lt;&gt;" ",G6&lt;&gt;"ERROR",H5&lt;&gt;" ", H5&lt;&gt;"ERROR"),G6+H5," ")</f>
-        <v>3</v>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I6" s="1">
         <f t="shared" si="1"/>
-        <v>0.75</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A7" s="1">
-        <v>2</v>
-      </c>
-      <c r="B7" s="4">
-        <v>44771</v>
-      </c>
-      <c r="C7" s="5">
-        <v>0.5625</v>
-      </c>
-      <c r="D7" s="4">
-        <v>44771</v>
-      </c>
-      <c r="E7" s="5">
-        <v>0.60416666666666663</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G7" s="6">
+      <c r="B7" s="4"/>
+      <c r="C7" s="5"/>
+      <c r="D7" s="4"/>
+      <c r="E7" s="5"/>
+      <c r="G7" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>0.99999999994179234</v>
-      </c>
-      <c r="H7" s="1">
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H7" s="1" t="str">
         <f t="shared" si="2"/>
-        <v>3.9999999999417923</v>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I7" s="1">
         <f t="shared" si="1"/>
-        <v>0.99999999994179234</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A8" s="1">
-        <v>2</v>
-      </c>
-      <c r="B8" s="4">
-        <v>44771</v>
-      </c>
-      <c r="C8" s="5">
-        <v>0.85416666666666663</v>
-      </c>
-      <c r="D8" s="4">
-        <v>44771</v>
-      </c>
-      <c r="E8" s="5">
-        <v>0.875</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G8" s="6">
+      <c r="B8" s="4"/>
+      <c r="C8" s="5"/>
+      <c r="D8" s="4"/>
+      <c r="E8" s="5"/>
+      <c r="G8" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>0.50000000005820766</v>
-      </c>
-      <c r="H8" s="1">
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H8" s="1" t="str">
         <f t="shared" si="2"/>
-        <v>4.5</v>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I8" s="1">
         <f t="shared" si="1"/>
-        <v>0.50000000005820766</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A9" s="1">
-        <v>2</v>
-      </c>
-      <c r="B9" s="4">
-        <v>44772</v>
-      </c>
-      <c r="C9" s="5">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="D9" s="4">
-        <v>44772</v>
-      </c>
-      <c r="E9" s="5">
-        <v>0.8125</v>
-      </c>
-      <c r="F9" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="G9" s="6">
+      <c r="B9" s="4"/>
+      <c r="C9" s="5"/>
+      <c r="D9" s="4"/>
+      <c r="E9" s="5"/>
+      <c r="G9" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>0.50000000005820766</v>
-      </c>
-      <c r="H9" s="1">
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H9" s="1" t="str">
         <f t="shared" si="2"/>
-        <v>5.0000000000582077</v>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I9" s="1">
         <f t="shared" si="1"/>
-        <v>0.50000000005820766</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.2">

</xml_diff>